<commit_message>
20250611 - update - sjudas - batidas
</commit_message>
<xml_diff>
--- a/1_apps/linux/sjudas/confinamento_batidas_trendline/dados_processados.xlsx
+++ b/1_apps/linux/sjudas/confinamento_batidas_trendline/dados_processados.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B466"/>
+  <dimension ref="A1:B1028"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4188,6 +4188,4502 @@
         <v>3.89</v>
       </c>
     </row>
+    <row r="467">
+      <c r="A467" t="n">
+        <v>29898</v>
+      </c>
+      <c r="B467" s="3" t="n">
+        <v>1.98</v>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="n">
+        <v>29899</v>
+      </c>
+      <c r="B468" s="3" t="n">
+        <v>1.81</v>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="n">
+        <v>29900</v>
+      </c>
+      <c r="B469" s="3" t="n">
+        <v>1.42</v>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="n">
+        <v>29901</v>
+      </c>
+      <c r="B470" s="3" t="n">
+        <v>1.88</v>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="n">
+        <v>29902</v>
+      </c>
+      <c r="B471" s="3" t="n">
+        <v>1.46</v>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="n">
+        <v>29903</v>
+      </c>
+      <c r="B472" s="3" t="n">
+        <v>2.04</v>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="n">
+        <v>29904</v>
+      </c>
+      <c r="B473" s="5" t="n">
+        <v>4.18</v>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="n">
+        <v>29905</v>
+      </c>
+      <c r="B474" s="3" t="n">
+        <v>1.44</v>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="n">
+        <v>29906</v>
+      </c>
+      <c r="B475" s="2" t="n">
+        <v>8.77</v>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="n">
+        <v>29907</v>
+      </c>
+      <c r="B476" s="3" t="n">
+        <v>2.36</v>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="n">
+        <v>29908</v>
+      </c>
+      <c r="B477" s="3" t="n">
+        <v>2.33</v>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="n">
+        <v>29909</v>
+      </c>
+      <c r="B478" s="5" t="n">
+        <v>3.66</v>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="n">
+        <v>29910</v>
+      </c>
+      <c r="B479" s="3" t="n">
+        <v>1.55</v>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="n">
+        <v>29911</v>
+      </c>
+      <c r="B480" s="5" t="n">
+        <v>3.33</v>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="n">
+        <v>29912</v>
+      </c>
+      <c r="B481" s="4" t="n">
+        <v>5.54</v>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="n">
+        <v>29913</v>
+      </c>
+      <c r="B482" s="3" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="n">
+        <v>29914</v>
+      </c>
+      <c r="B483" s="3" t="n">
+        <v>2.58</v>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="n">
+        <v>29915</v>
+      </c>
+      <c r="B484" s="2" t="n">
+        <v>10.2</v>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="n">
+        <v>29916</v>
+      </c>
+      <c r="B485" s="3" t="n">
+        <v>2.47</v>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="n">
+        <v>29917</v>
+      </c>
+      <c r="B486" s="3" t="n">
+        <v>1.74</v>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="n">
+        <v>29918</v>
+      </c>
+      <c r="B487" s="3" t="n">
+        <v>2.69</v>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="n">
+        <v>29919</v>
+      </c>
+      <c r="B488" s="3" t="n">
+        <v>1.45</v>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="n">
+        <v>29920</v>
+      </c>
+      <c r="B489" s="3" t="n">
+        <v>0.77</v>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="n">
+        <v>29921</v>
+      </c>
+      <c r="B490" s="3" t="n">
+        <v>1.74</v>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="n">
+        <v>29922</v>
+      </c>
+      <c r="B491" s="3" t="n">
+        <v>2.34</v>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="n">
+        <v>29923</v>
+      </c>
+      <c r="B492" s="3" t="n">
+        <v>2.27</v>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="n">
+        <v>29924</v>
+      </c>
+      <c r="B493" s="3" t="n">
+        <v>1.37</v>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="n">
+        <v>29925</v>
+      </c>
+      <c r="B494" s="3" t="n">
+        <v>1.88</v>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="n">
+        <v>29926</v>
+      </c>
+      <c r="B495" s="4" t="n">
+        <v>5.48</v>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="n">
+        <v>29927</v>
+      </c>
+      <c r="B496" s="5" t="n">
+        <v>3.64</v>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="n">
+        <v>29928</v>
+      </c>
+      <c r="B497" s="3" t="n">
+        <v>2.56</v>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="n">
+        <v>29929</v>
+      </c>
+      <c r="B498" s="3" t="n">
+        <v>2.76</v>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="n">
+        <v>29930</v>
+      </c>
+      <c r="B499" s="2" t="n">
+        <v>12.07</v>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="n">
+        <v>29931</v>
+      </c>
+      <c r="B500" s="4" t="n">
+        <v>5.52</v>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="n">
+        <v>29932</v>
+      </c>
+      <c r="B501" s="3" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="n">
+        <v>29933</v>
+      </c>
+      <c r="B502" s="3" t="n">
+        <v>0.73</v>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="n">
+        <v>29934</v>
+      </c>
+      <c r="B503" s="3" t="n">
+        <v>1.54</v>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="n">
+        <v>29935</v>
+      </c>
+      <c r="B504" s="3" t="n">
+        <v>1.23</v>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="n">
+        <v>29936</v>
+      </c>
+      <c r="B505" s="3" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="n">
+        <v>29937</v>
+      </c>
+      <c r="B506" s="3" t="n">
+        <v>0.93</v>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="n">
+        <v>29938</v>
+      </c>
+      <c r="B507" s="5" t="n">
+        <v>4.98</v>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="n">
+        <v>29939</v>
+      </c>
+      <c r="B508" s="4" t="n">
+        <v>6.44</v>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="n">
+        <v>29940</v>
+      </c>
+      <c r="B509" s="5" t="n">
+        <v>4.08</v>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="n">
+        <v>29941</v>
+      </c>
+      <c r="B510" s="2" t="n">
+        <v>9.08</v>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="n">
+        <v>29942</v>
+      </c>
+      <c r="B511" s="3" t="n">
+        <v>2.02</v>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="n">
+        <v>29943</v>
+      </c>
+      <c r="B512" s="3" t="n">
+        <v>2.35</v>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="n">
+        <v>29944</v>
+      </c>
+      <c r="B513" s="5" t="n">
+        <v>3.13</v>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="n">
+        <v>29945</v>
+      </c>
+      <c r="B514" s="5" t="n">
+        <v>3.04</v>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="n">
+        <v>29946</v>
+      </c>
+      <c r="B515" s="3" t="n">
+        <v>1.67</v>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="n">
+        <v>29947</v>
+      </c>
+      <c r="B516" s="5" t="n">
+        <v>4.41</v>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="n">
+        <v>29948</v>
+      </c>
+      <c r="B517" s="5" t="n">
+        <v>3.3</v>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="n">
+        <v>29949</v>
+      </c>
+      <c r="B518" s="3" t="n">
+        <v>2.24</v>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="n">
+        <v>29950</v>
+      </c>
+      <c r="B519" s="2" t="n">
+        <v>10.75</v>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="n">
+        <v>29951</v>
+      </c>
+      <c r="B520" s="5" t="n">
+        <v>4.73</v>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="n">
+        <v>29952</v>
+      </c>
+      <c r="B521" s="3" t="n">
+        <v>2.51</v>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="n">
+        <v>29953</v>
+      </c>
+      <c r="B522" s="5" t="n">
+        <v>3.72</v>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="n">
+        <v>29954</v>
+      </c>
+      <c r="B523" s="4" t="n">
+        <v>6.45</v>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="n">
+        <v>29955</v>
+      </c>
+      <c r="B524" s="3" t="n">
+        <v>2.08</v>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="n">
+        <v>29956</v>
+      </c>
+      <c r="B525" s="3" t="n">
+        <v>1.72</v>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="n">
+        <v>29957</v>
+      </c>
+      <c r="B526" s="2" t="n">
+        <v>14.76</v>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="n">
+        <v>29958</v>
+      </c>
+      <c r="B527" s="5" t="n">
+        <v>3.87</v>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="n">
+        <v>29959</v>
+      </c>
+      <c r="B528" s="2" t="n">
+        <v>7.94</v>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="n">
+        <v>29960</v>
+      </c>
+      <c r="B529" s="5" t="n">
+        <v>3.72</v>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="n">
+        <v>29961</v>
+      </c>
+      <c r="B530" s="3" t="n">
+        <v>1.7</v>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="n">
+        <v>29962</v>
+      </c>
+      <c r="B531" s="5" t="n">
+        <v>4.42</v>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="n">
+        <v>29963</v>
+      </c>
+      <c r="B532" s="5" t="n">
+        <v>3.35</v>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="n">
+        <v>29964</v>
+      </c>
+      <c r="B533" s="4" t="n">
+        <v>6.82</v>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="n">
+        <v>29965</v>
+      </c>
+      <c r="B534" s="5" t="n">
+        <v>3.64</v>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="n">
+        <v>29966</v>
+      </c>
+      <c r="B535" s="2" t="n">
+        <v>19.69</v>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="n">
+        <v>29967</v>
+      </c>
+      <c r="B536" s="4" t="n">
+        <v>5.49</v>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="n">
+        <v>29968</v>
+      </c>
+      <c r="B537" s="4" t="n">
+        <v>6.91</v>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="n">
+        <v>29969</v>
+      </c>
+      <c r="B538" s="4" t="n">
+        <v>5.28</v>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="n">
+        <v>29970</v>
+      </c>
+      <c r="B539" s="5" t="n">
+        <v>3.42</v>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="n">
+        <v>29971</v>
+      </c>
+      <c r="B540" s="3" t="n">
+        <v>2.46</v>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="n">
+        <v>29972</v>
+      </c>
+      <c r="B541" s="2" t="n">
+        <v>8.48</v>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="n">
+        <v>29973</v>
+      </c>
+      <c r="B542" s="3" t="n">
+        <v>1.17</v>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="n">
+        <v>29974</v>
+      </c>
+      <c r="B543" s="4" t="n">
+        <v>5.06</v>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="n">
+        <v>29975</v>
+      </c>
+      <c r="B544" s="5" t="n">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="n">
+        <v>29976</v>
+      </c>
+      <c r="B545" s="5" t="n">
+        <v>4.87</v>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="n">
+        <v>29977</v>
+      </c>
+      <c r="B546" s="5" t="n">
+        <v>3.76</v>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="n">
+        <v>29978</v>
+      </c>
+      <c r="B547" s="3" t="n">
+        <v>2.27</v>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="n">
+        <v>29979</v>
+      </c>
+      <c r="B548" s="2" t="n">
+        <v>8.16</v>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="n">
+        <v>29980</v>
+      </c>
+      <c r="B549" s="2" t="n">
+        <v>16.61</v>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="n">
+        <v>29981</v>
+      </c>
+      <c r="B550" s="5" t="n">
+        <v>3.29</v>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="n">
+        <v>29982</v>
+      </c>
+      <c r="B551" s="3" t="n">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="n">
+        <v>29983</v>
+      </c>
+      <c r="B552" s="4" t="n">
+        <v>6.88</v>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="n">
+        <v>29984</v>
+      </c>
+      <c r="B553" s="5" t="n">
+        <v>4.02</v>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="n">
+        <v>29985</v>
+      </c>
+      <c r="B554" s="3" t="n">
+        <v>1.29</v>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="n">
+        <v>29986</v>
+      </c>
+      <c r="B555" s="5" t="n">
+        <v>3.98</v>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="n">
+        <v>29987</v>
+      </c>
+      <c r="B556" s="2" t="n">
+        <v>15.36</v>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="n">
+        <v>29988</v>
+      </c>
+      <c r="B557" s="3" t="n">
+        <v>1.92</v>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="n">
+        <v>29989</v>
+      </c>
+      <c r="B558" s="3" t="n">
+        <v>1.92</v>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="n">
+        <v>29990</v>
+      </c>
+      <c r="B559" s="3" t="n">
+        <v>1.92</v>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="n">
+        <v>29991</v>
+      </c>
+      <c r="B560" s="2" t="n">
+        <v>32.04</v>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="n">
+        <v>29992</v>
+      </c>
+      <c r="B561" s="3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="n">
+        <v>29993</v>
+      </c>
+      <c r="B562" s="3" t="n">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="n">
+        <v>29994</v>
+      </c>
+      <c r="B563" s="3" t="n">
+        <v>1.41</v>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="n">
+        <v>29995</v>
+      </c>
+      <c r="B564" s="2" t="n">
+        <v>8.08</v>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="n">
+        <v>29996</v>
+      </c>
+      <c r="B565" s="3" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="n">
+        <v>29997</v>
+      </c>
+      <c r="B566" s="5" t="n">
+        <v>3.11</v>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="n">
+        <v>29998</v>
+      </c>
+      <c r="B567" s="2" t="n">
+        <v>9.91</v>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="n">
+        <v>29999</v>
+      </c>
+      <c r="B568" s="4" t="n">
+        <v>5.2</v>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="n">
+        <v>30000</v>
+      </c>
+      <c r="B569" s="3" t="n">
+        <v>2.91</v>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="n">
+        <v>30001</v>
+      </c>
+      <c r="B570" s="3" t="n">
+        <v>1.63</v>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="n">
+        <v>30002</v>
+      </c>
+      <c r="B571" s="4" t="n">
+        <v>6.86</v>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="n">
+        <v>30003</v>
+      </c>
+      <c r="B572" s="5" t="n">
+        <v>4.02</v>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="n">
+        <v>30004</v>
+      </c>
+      <c r="B573" s="5" t="n">
+        <v>4.65</v>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="n">
+        <v>30005</v>
+      </c>
+      <c r="B574" s="3" t="n">
+        <v>1.76</v>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="n">
+        <v>30006</v>
+      </c>
+      <c r="B575" s="3" t="n">
+        <v>0.72</v>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="n">
+        <v>30007</v>
+      </c>
+      <c r="B576" s="3" t="n">
+        <v>1.06</v>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="n">
+        <v>30008</v>
+      </c>
+      <c r="B577" s="3" t="n">
+        <v>1.21</v>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="n">
+        <v>30009</v>
+      </c>
+      <c r="B578" s="3" t="n">
+        <v>2.83</v>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="n">
+        <v>30010</v>
+      </c>
+      <c r="B579" s="4" t="n">
+        <v>5.75</v>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="n">
+        <v>30011</v>
+      </c>
+      <c r="B580" s="5" t="n">
+        <v>3.71</v>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="n">
+        <v>30012</v>
+      </c>
+      <c r="B581" s="2" t="n">
+        <v>7.73</v>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="n">
+        <v>30013</v>
+      </c>
+      <c r="B582" s="5" t="n">
+        <v>4.25</v>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="n">
+        <v>30014</v>
+      </c>
+      <c r="B583" s="4" t="n">
+        <v>5.54</v>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" t="n">
+        <v>30015</v>
+      </c>
+      <c r="B584" s="3" t="n">
+        <v>1.01</v>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="n">
+        <v>30016</v>
+      </c>
+      <c r="B585" s="4" t="n">
+        <v>5.51</v>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="n">
+        <v>30017</v>
+      </c>
+      <c r="B586" s="3" t="n">
+        <v>2.65</v>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="n">
+        <v>30018</v>
+      </c>
+      <c r="B587" s="3" t="n">
+        <v>2.49</v>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="n">
+        <v>30019</v>
+      </c>
+      <c r="B588" s="4" t="n">
+        <v>5.26</v>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="n">
+        <v>30020</v>
+      </c>
+      <c r="B589" s="3" t="n">
+        <v>1.04</v>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="n">
+        <v>30021</v>
+      </c>
+      <c r="B590" s="4" t="n">
+        <v>6.98</v>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="n">
+        <v>30022</v>
+      </c>
+      <c r="B591" s="4" t="n">
+        <v>5.06</v>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="n">
+        <v>30023</v>
+      </c>
+      <c r="B592" s="2" t="n">
+        <v>8.460000000000001</v>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="n">
+        <v>30024</v>
+      </c>
+      <c r="B593" s="3" t="n">
+        <v>2.68</v>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="n">
+        <v>30025</v>
+      </c>
+      <c r="B594" s="3" t="n">
+        <v>1.88</v>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="n">
+        <v>30026</v>
+      </c>
+      <c r="B595" s="2" t="n">
+        <v>17.66</v>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="n">
+        <v>30027</v>
+      </c>
+      <c r="B596" s="5" t="n">
+        <v>3.87</v>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="n">
+        <v>30028</v>
+      </c>
+      <c r="B597" s="3" t="n">
+        <v>1.41</v>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="n">
+        <v>30029</v>
+      </c>
+      <c r="B598" s="2" t="n">
+        <v>8.09</v>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="n">
+        <v>30030</v>
+      </c>
+      <c r="B599" s="3" t="n">
+        <v>2.12</v>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="n">
+        <v>30031</v>
+      </c>
+      <c r="B600" s="2" t="n">
+        <v>11.53</v>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="n">
+        <v>30032</v>
+      </c>
+      <c r="B601" s="3" t="n">
+        <v>1.7</v>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="n">
+        <v>30033</v>
+      </c>
+      <c r="B602" s="3" t="n">
+        <v>2.55</v>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" t="n">
+        <v>30034</v>
+      </c>
+      <c r="B603" s="3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="n">
+        <v>30035</v>
+      </c>
+      <c r="B604" s="3" t="n">
+        <v>2.22</v>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="n">
+        <v>30036</v>
+      </c>
+      <c r="B605" s="4" t="n">
+        <v>5.39</v>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="n">
+        <v>30037</v>
+      </c>
+      <c r="B606" s="3" t="n">
+        <v>1.87</v>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="n">
+        <v>30038</v>
+      </c>
+      <c r="B607" s="3" t="n">
+        <v>1.22</v>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="n">
+        <v>30039</v>
+      </c>
+      <c r="B608" s="5" t="n">
+        <v>4.77</v>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="n">
+        <v>30040</v>
+      </c>
+      <c r="B609" s="3" t="n">
+        <v>0.74</v>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" t="n">
+        <v>30041</v>
+      </c>
+      <c r="B610" s="3" t="n">
+        <v>2.27</v>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" t="n">
+        <v>30042</v>
+      </c>
+      <c r="B611" s="3" t="n">
+        <v>2.74</v>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" t="n">
+        <v>30043</v>
+      </c>
+      <c r="B612" s="4" t="n">
+        <v>6.55</v>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" t="n">
+        <v>30044</v>
+      </c>
+      <c r="B613" s="3" t="n">
+        <v>2.62</v>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" t="n">
+        <v>30045</v>
+      </c>
+      <c r="B614" s="3" t="n">
+        <v>2.49</v>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="n">
+        <v>30046</v>
+      </c>
+      <c r="B615" s="5" t="n">
+        <v>3.64</v>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" t="n">
+        <v>30048</v>
+      </c>
+      <c r="B616" s="3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" t="n">
+        <v>30049</v>
+      </c>
+      <c r="B617" s="3" t="n">
+        <v>2.57</v>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="n">
+        <v>30050</v>
+      </c>
+      <c r="B618" s="3" t="n">
+        <v>0.96</v>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" t="n">
+        <v>30051</v>
+      </c>
+      <c r="B619" s="4" t="n">
+        <v>5.37</v>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="n">
+        <v>30052</v>
+      </c>
+      <c r="B620" s="5" t="n">
+        <v>3.49</v>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="n">
+        <v>30053</v>
+      </c>
+      <c r="B621" s="5" t="n">
+        <v>4.45</v>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="n">
+        <v>30054</v>
+      </c>
+      <c r="B622" s="3" t="n">
+        <v>1.12</v>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="n">
+        <v>30055</v>
+      </c>
+      <c r="B623" s="5" t="n">
+        <v>3.27</v>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="n">
+        <v>30056</v>
+      </c>
+      <c r="B624" s="3" t="n">
+        <v>1.58</v>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" t="n">
+        <v>30057</v>
+      </c>
+      <c r="B625" s="3" t="n">
+        <v>2.94</v>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" t="n">
+        <v>30058</v>
+      </c>
+      <c r="B626" s="5" t="n">
+        <v>3.95</v>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" t="n">
+        <v>30059</v>
+      </c>
+      <c r="B627" s="5" t="n">
+        <v>3.33</v>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" t="n">
+        <v>30060</v>
+      </c>
+      <c r="B628" s="3" t="n">
+        <v>2.62</v>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" t="n">
+        <v>30061</v>
+      </c>
+      <c r="B629" s="5" t="n">
+        <v>3.07</v>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" t="n">
+        <v>30062</v>
+      </c>
+      <c r="B630" s="5" t="n">
+        <v>4.46</v>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="n">
+        <v>30063</v>
+      </c>
+      <c r="B631" s="3" t="n">
+        <v>1.02</v>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" t="n">
+        <v>30064</v>
+      </c>
+      <c r="B632" s="3" t="n">
+        <v>0.86</v>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" t="n">
+        <v>30065</v>
+      </c>
+      <c r="B633" s="5" t="n">
+        <v>4.84</v>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" t="n">
+        <v>30066</v>
+      </c>
+      <c r="B634" s="2" t="n">
+        <v>108.05</v>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" t="n">
+        <v>30067</v>
+      </c>
+      <c r="B635" s="3" t="n">
+        <v>1.7</v>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="n">
+        <v>30068</v>
+      </c>
+      <c r="B636" s="3" t="n">
+        <v>2.44</v>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="n">
+        <v>30069</v>
+      </c>
+      <c r="B637" s="3" t="n">
+        <v>2.82</v>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="n">
+        <v>30070</v>
+      </c>
+      <c r="B638" s="3" t="n">
+        <v>1.69</v>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="n">
+        <v>30071</v>
+      </c>
+      <c r="B639" s="3" t="n">
+        <v>1.68</v>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="n">
+        <v>30072</v>
+      </c>
+      <c r="B640" s="5" t="n">
+        <v>4.91</v>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="n">
+        <v>30073</v>
+      </c>
+      <c r="B641" s="4" t="n">
+        <v>5.78</v>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="n">
+        <v>30074</v>
+      </c>
+      <c r="B642" s="3" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="n">
+        <v>30075</v>
+      </c>
+      <c r="B643" s="2" t="n">
+        <v>7.47</v>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="n">
+        <v>30076</v>
+      </c>
+      <c r="B644" s="5" t="n">
+        <v>3.15</v>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="n">
+        <v>30077</v>
+      </c>
+      <c r="B645" s="3" t="n">
+        <v>1.08</v>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" t="n">
+        <v>30078</v>
+      </c>
+      <c r="B646" s="4" t="n">
+        <v>5.65</v>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="n">
+        <v>30079</v>
+      </c>
+      <c r="B647" s="5" t="n">
+        <v>4.11</v>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" t="n">
+        <v>30080</v>
+      </c>
+      <c r="B648" s="3" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="n">
+        <v>30081</v>
+      </c>
+      <c r="B649" s="5" t="n">
+        <v>3.42</v>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="n">
+        <v>30082</v>
+      </c>
+      <c r="B650" s="3" t="n">
+        <v>2.74</v>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="n">
+        <v>30083</v>
+      </c>
+      <c r="B651" s="5" t="n">
+        <v>3.97</v>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="n">
+        <v>30084</v>
+      </c>
+      <c r="B652" s="3" t="n">
+        <v>1.02</v>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" t="n">
+        <v>30085</v>
+      </c>
+      <c r="B653" s="3" t="n">
+        <v>1.58</v>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="n">
+        <v>30086</v>
+      </c>
+      <c r="B654" s="3" t="n">
+        <v>2.03</v>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" t="n">
+        <v>30087</v>
+      </c>
+      <c r="B655" s="3" t="n">
+        <v>1.71</v>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" t="n">
+        <v>30088</v>
+      </c>
+      <c r="B656" s="5" t="n">
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="n">
+        <v>30089</v>
+      </c>
+      <c r="B657" s="3" t="n">
+        <v>2.47</v>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="n">
+        <v>30090</v>
+      </c>
+      <c r="B658" s="5" t="n">
+        <v>3.73</v>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" t="n">
+        <v>30091</v>
+      </c>
+      <c r="B659" s="5" t="n">
+        <v>3.27</v>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" t="n">
+        <v>30092</v>
+      </c>
+      <c r="B660" s="3" t="n">
+        <v>0.26</v>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" t="n">
+        <v>30093</v>
+      </c>
+      <c r="B661" s="5" t="n">
+        <v>3.46</v>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="n">
+        <v>30094</v>
+      </c>
+      <c r="B662" s="3" t="n">
+        <v>1.46</v>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="n">
+        <v>30095</v>
+      </c>
+      <c r="B663" s="5" t="n">
+        <v>4.26</v>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="n">
+        <v>30096</v>
+      </c>
+      <c r="B664" s="3" t="n">
+        <v>0.99</v>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="n">
+        <v>30097</v>
+      </c>
+      <c r="B665" s="4" t="n">
+        <v>6.86</v>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="n">
+        <v>30098</v>
+      </c>
+      <c r="B666" s="5" t="n">
+        <v>3.27</v>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" t="n">
+        <v>30099</v>
+      </c>
+      <c r="B667" s="3" t="n">
+        <v>2.64</v>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="n">
+        <v>30100</v>
+      </c>
+      <c r="B668" s="3" t="n">
+        <v>1.56</v>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="n">
+        <v>30101</v>
+      </c>
+      <c r="B669" s="5" t="n">
+        <v>3.15</v>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="n">
+        <v>30102</v>
+      </c>
+      <c r="B670" s="5" t="n">
+        <v>3.88</v>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="n">
+        <v>30103</v>
+      </c>
+      <c r="B671" s="5" t="n">
+        <v>3.24</v>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="n">
+        <v>30104</v>
+      </c>
+      <c r="B672" s="5" t="n">
+        <v>3.02</v>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="n">
+        <v>30105</v>
+      </c>
+      <c r="B673" s="5" t="n">
+        <v>3.56</v>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="n">
+        <v>30106</v>
+      </c>
+      <c r="B674" s="5" t="n">
+        <v>3.66</v>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="n">
+        <v>30107</v>
+      </c>
+      <c r="B675" s="2" t="n">
+        <v>9.19</v>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="n">
+        <v>30108</v>
+      </c>
+      <c r="B676" s="3" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="n">
+        <v>30109</v>
+      </c>
+      <c r="B677" s="3" t="n">
+        <v>2.84</v>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="n">
+        <v>30110</v>
+      </c>
+      <c r="B678" s="5" t="n">
+        <v>4.37</v>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="n">
+        <v>30111</v>
+      </c>
+      <c r="B679" s="3" t="n">
+        <v>2.22</v>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="n">
+        <v>30112</v>
+      </c>
+      <c r="B680" s="5" t="n">
+        <v>3.55</v>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="n">
+        <v>30113</v>
+      </c>
+      <c r="B681" s="3" t="n">
+        <v>1.55</v>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="n">
+        <v>30114</v>
+      </c>
+      <c r="B682" s="3" t="n">
+        <v>1.08</v>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="n">
+        <v>30115</v>
+      </c>
+      <c r="B683" s="2" t="n">
+        <v>10.26</v>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" t="n">
+        <v>30116</v>
+      </c>
+      <c r="B684" s="3" t="n">
+        <v>1.84</v>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" t="n">
+        <v>30117</v>
+      </c>
+      <c r="B685" s="3" t="n">
+        <v>2.33</v>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" t="n">
+        <v>30118</v>
+      </c>
+      <c r="B686" s="3" t="n">
+        <v>2.76</v>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" t="n">
+        <v>30119</v>
+      </c>
+      <c r="B687" s="3" t="n">
+        <v>1.79</v>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" t="n">
+        <v>30120</v>
+      </c>
+      <c r="B688" s="5" t="n">
+        <v>3.63</v>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" t="n">
+        <v>30121</v>
+      </c>
+      <c r="B689" s="3" t="n">
+        <v>1.19</v>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" t="n">
+        <v>30122</v>
+      </c>
+      <c r="B690" s="5" t="n">
+        <v>4.97</v>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" t="n">
+        <v>30123</v>
+      </c>
+      <c r="B691" s="5" t="n">
+        <v>4.88</v>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" t="n">
+        <v>30124</v>
+      </c>
+      <c r="B692" s="2" t="n">
+        <v>25.32</v>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" t="n">
+        <v>30125</v>
+      </c>
+      <c r="B693" s="2" t="n">
+        <v>9.460000000000001</v>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" t="n">
+        <v>30126</v>
+      </c>
+      <c r="B694" s="5" t="n">
+        <v>3.51</v>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" t="n">
+        <v>30127</v>
+      </c>
+      <c r="B695" s="5" t="n">
+        <v>4.93</v>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" t="n">
+        <v>30128</v>
+      </c>
+      <c r="B696" s="5" t="n">
+        <v>4.87</v>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" t="n">
+        <v>30129</v>
+      </c>
+      <c r="B697" s="3" t="n">
+        <v>1.41</v>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" t="n">
+        <v>30130</v>
+      </c>
+      <c r="B698" s="3" t="n">
+        <v>1.23</v>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" t="n">
+        <v>30131</v>
+      </c>
+      <c r="B699" s="3" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" t="n">
+        <v>30132</v>
+      </c>
+      <c r="B700" s="3" t="n">
+        <v>1.88</v>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" t="n">
+        <v>30133</v>
+      </c>
+      <c r="B701" s="4" t="n">
+        <v>5.96</v>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" t="n">
+        <v>30134</v>
+      </c>
+      <c r="B702" s="4" t="n">
+        <v>6.22</v>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" t="n">
+        <v>30135</v>
+      </c>
+      <c r="B703" s="3" t="n">
+        <v>2.81</v>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" t="n">
+        <v>30136</v>
+      </c>
+      <c r="B704" s="2" t="n">
+        <v>17.39</v>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" t="n">
+        <v>30137</v>
+      </c>
+      <c r="B705" s="3" t="n">
+        <v>1.81</v>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" t="n">
+        <v>30138</v>
+      </c>
+      <c r="B706" s="4" t="n">
+        <v>5.57</v>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" t="n">
+        <v>30139</v>
+      </c>
+      <c r="B707" s="2" t="n">
+        <v>7.12</v>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" t="n">
+        <v>30140</v>
+      </c>
+      <c r="B708" s="4" t="n">
+        <v>5.71</v>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" t="n">
+        <v>30141</v>
+      </c>
+      <c r="B709" s="3" t="n">
+        <v>1.64</v>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" t="n">
+        <v>30142</v>
+      </c>
+      <c r="B710" s="5" t="n">
+        <v>3.46</v>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" t="n">
+        <v>30143</v>
+      </c>
+      <c r="B711" s="2" t="n">
+        <v>9.93</v>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" t="n">
+        <v>30144</v>
+      </c>
+      <c r="B712" s="3" t="n">
+        <v>1.65</v>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" t="n">
+        <v>30145</v>
+      </c>
+      <c r="B713" s="5" t="n">
+        <v>3.12</v>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" t="n">
+        <v>30146</v>
+      </c>
+      <c r="B714" s="5" t="n">
+        <v>3.37</v>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" t="n">
+        <v>30147</v>
+      </c>
+      <c r="B715" s="5" t="n">
+        <v>4.25</v>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" t="n">
+        <v>30148</v>
+      </c>
+      <c r="B716" s="5" t="n">
+        <v>4.32</v>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" t="n">
+        <v>30149</v>
+      </c>
+      <c r="B717" s="3" t="n">
+        <v>0.28</v>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" t="n">
+        <v>30150</v>
+      </c>
+      <c r="B718" s="3" t="n">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" t="n">
+        <v>30151</v>
+      </c>
+      <c r="B719" s="3" t="n">
+        <v>2.78</v>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" t="n">
+        <v>30152</v>
+      </c>
+      <c r="B720" s="5" t="n">
+        <v>4.94</v>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" t="n">
+        <v>30153</v>
+      </c>
+      <c r="B721" s="2" t="n">
+        <v>11.02</v>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" t="n">
+        <v>30154</v>
+      </c>
+      <c r="B722" s="3" t="n">
+        <v>2.35</v>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" t="n">
+        <v>30155</v>
+      </c>
+      <c r="B723" s="5" t="n">
+        <v>3.19</v>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" t="n">
+        <v>30156</v>
+      </c>
+      <c r="B724" s="5" t="n">
+        <v>4.24</v>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" t="n">
+        <v>30157</v>
+      </c>
+      <c r="B725" s="3" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" t="n">
+        <v>30158</v>
+      </c>
+      <c r="B726" s="3" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" t="n">
+        <v>30159</v>
+      </c>
+      <c r="B727" s="3" t="n">
+        <v>1.08</v>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" t="n">
+        <v>30160</v>
+      </c>
+      <c r="B728" s="3" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" t="n">
+        <v>30161</v>
+      </c>
+      <c r="B729" s="3" t="n">
+        <v>0.98</v>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" t="n">
+        <v>30162</v>
+      </c>
+      <c r="B730" s="3" t="n">
+        <v>2.63</v>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" t="n">
+        <v>30163</v>
+      </c>
+      <c r="B731" s="5" t="n">
+        <v>3.32</v>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" t="n">
+        <v>30164</v>
+      </c>
+      <c r="B732" s="5" t="n">
+        <v>3.57</v>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" t="n">
+        <v>30165</v>
+      </c>
+      <c r="B733" s="5" t="n">
+        <v>3.55</v>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" t="n">
+        <v>30166</v>
+      </c>
+      <c r="B734" s="3" t="n">
+        <v>2.42</v>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" t="n">
+        <v>30167</v>
+      </c>
+      <c r="B735" s="5" t="n">
+        <v>4.79</v>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" t="n">
+        <v>30168</v>
+      </c>
+      <c r="B736" s="5" t="n">
+        <v>4.41</v>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" t="n">
+        <v>30169</v>
+      </c>
+      <c r="B737" s="5" t="n">
+        <v>4.57</v>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" t="n">
+        <v>30170</v>
+      </c>
+      <c r="B738" s="3" t="n">
+        <v>1.32</v>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" t="n">
+        <v>30171</v>
+      </c>
+      <c r="B739" s="4" t="n">
+        <v>6.59</v>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" t="n">
+        <v>30172</v>
+      </c>
+      <c r="B740" s="3" t="n">
+        <v>1.65</v>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" t="n">
+        <v>30173</v>
+      </c>
+      <c r="B741" s="5" t="n">
+        <v>3.79</v>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" t="n">
+        <v>30174</v>
+      </c>
+      <c r="B742" s="3" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" t="n">
+        <v>30175</v>
+      </c>
+      <c r="B743" s="5" t="n">
+        <v>3.86</v>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" t="n">
+        <v>30176</v>
+      </c>
+      <c r="B744" s="2" t="n">
+        <v>8.779999999999999</v>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" t="n">
+        <v>30177</v>
+      </c>
+      <c r="B745" s="3" t="n">
+        <v>2.52</v>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" t="n">
+        <v>30178</v>
+      </c>
+      <c r="B746" s="2" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" t="n">
+        <v>30179</v>
+      </c>
+      <c r="B747" s="3" t="n">
+        <v>2.62</v>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" t="n">
+        <v>30180</v>
+      </c>
+      <c r="B748" s="2" t="n">
+        <v>8.199999999999999</v>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" t="n">
+        <v>30181</v>
+      </c>
+      <c r="B749" s="2" t="n">
+        <v>8.970000000000001</v>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" t="n">
+        <v>30182</v>
+      </c>
+      <c r="B750" s="3" t="n">
+        <v>1.68</v>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" t="n">
+        <v>30183</v>
+      </c>
+      <c r="B751" s="3" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" t="n">
+        <v>30184</v>
+      </c>
+      <c r="B752" s="5" t="n">
+        <v>3.33</v>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" t="n">
+        <v>30185</v>
+      </c>
+      <c r="B753" s="3" t="n">
+        <v>1.97</v>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" t="n">
+        <v>30186</v>
+      </c>
+      <c r="B754" s="3" t="n">
+        <v>1.26</v>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" t="n">
+        <v>30187</v>
+      </c>
+      <c r="B755" s="4" t="n">
+        <v>6.9</v>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" t="n">
+        <v>30188</v>
+      </c>
+      <c r="B756" s="4" t="n">
+        <v>5.76</v>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" t="n">
+        <v>30189</v>
+      </c>
+      <c r="B757" s="2" t="n">
+        <v>11.19</v>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" t="n">
+        <v>30190</v>
+      </c>
+      <c r="B758" s="3" t="n">
+        <v>2.7</v>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" t="n">
+        <v>30191</v>
+      </c>
+      <c r="B759" s="3" t="n">
+        <v>1.65</v>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" t="n">
+        <v>30192</v>
+      </c>
+      <c r="B760" s="3" t="n">
+        <v>0.83</v>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" t="n">
+        <v>30193</v>
+      </c>
+      <c r="B761" s="3" t="n">
+        <v>2.86</v>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" t="n">
+        <v>30194</v>
+      </c>
+      <c r="B762" s="3" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" t="n">
+        <v>30195</v>
+      </c>
+      <c r="B763" s="3" t="n">
+        <v>1.36</v>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" t="n">
+        <v>30196</v>
+      </c>
+      <c r="B764" s="3" t="n">
+        <v>1.56</v>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" t="n">
+        <v>30197</v>
+      </c>
+      <c r="B765" s="2" t="n">
+        <v>10.2</v>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" t="n">
+        <v>30198</v>
+      </c>
+      <c r="B766" s="3" t="n">
+        <v>0.66</v>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" t="n">
+        <v>30199</v>
+      </c>
+      <c r="B767" s="4" t="n">
+        <v>6.82</v>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" t="n">
+        <v>30200</v>
+      </c>
+      <c r="B768" s="3" t="n">
+        <v>2.49</v>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" t="n">
+        <v>30201</v>
+      </c>
+      <c r="B769" s="5" t="n">
+        <v>4.16</v>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" t="n">
+        <v>30202</v>
+      </c>
+      <c r="B770" s="3" t="n">
+        <v>1.74</v>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" t="n">
+        <v>30203</v>
+      </c>
+      <c r="B771" s="5" t="n">
+        <v>3.44</v>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" t="n">
+        <v>30204</v>
+      </c>
+      <c r="B772" s="4" t="n">
+        <v>5.84</v>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" t="n">
+        <v>30205</v>
+      </c>
+      <c r="B773" s="5" t="n">
+        <v>3.16</v>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" t="n">
+        <v>30206</v>
+      </c>
+      <c r="B774" s="3" t="n">
+        <v>2.78</v>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" t="n">
+        <v>30207</v>
+      </c>
+      <c r="B775" s="5" t="n">
+        <v>4.41</v>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" t="n">
+        <v>30208</v>
+      </c>
+      <c r="B776" s="5" t="n">
+        <v>3.3</v>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" t="n">
+        <v>30209</v>
+      </c>
+      <c r="B777" s="5" t="n">
+        <v>4.6</v>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" t="n">
+        <v>30210</v>
+      </c>
+      <c r="B778" s="5" t="n">
+        <v>3.73</v>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" t="n">
+        <v>30211</v>
+      </c>
+      <c r="B779" s="3" t="n">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" t="n">
+        <v>30212</v>
+      </c>
+      <c r="B780" s="5" t="n">
+        <v>4.82</v>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" t="n">
+        <v>30213</v>
+      </c>
+      <c r="B781" s="2" t="n">
+        <v>17.93</v>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" t="n">
+        <v>30214</v>
+      </c>
+      <c r="B782" s="4" t="n">
+        <v>6.75</v>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" t="n">
+        <v>30215</v>
+      </c>
+      <c r="B783" s="3" t="n">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" t="n">
+        <v>30216</v>
+      </c>
+      <c r="B784" s="3" t="n">
+        <v>1.47</v>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" t="n">
+        <v>30217</v>
+      </c>
+      <c r="B785" s="5" t="n">
+        <v>4.02</v>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" t="n">
+        <v>30218</v>
+      </c>
+      <c r="B786" s="3" t="n">
+        <v>2.52</v>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" t="n">
+        <v>30219</v>
+      </c>
+      <c r="B787" s="5" t="n">
+        <v>3.11</v>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" t="n">
+        <v>30220</v>
+      </c>
+      <c r="B788" s="3" t="n">
+        <v>1.96</v>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" t="n">
+        <v>30221</v>
+      </c>
+      <c r="B789" s="3" t="n">
+        <v>2.69</v>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" t="n">
+        <v>30222</v>
+      </c>
+      <c r="B790" s="3" t="n">
+        <v>1.38</v>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" t="n">
+        <v>30223</v>
+      </c>
+      <c r="B791" s="2" t="n">
+        <v>9.609999999999999</v>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" t="n">
+        <v>30224</v>
+      </c>
+      <c r="B792" s="3" t="n">
+        <v>2.86</v>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" t="n">
+        <v>30225</v>
+      </c>
+      <c r="B793" s="4" t="n">
+        <v>5.11</v>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" t="n">
+        <v>30226</v>
+      </c>
+      <c r="B794" s="2" t="n">
+        <v>8.65</v>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" t="n">
+        <v>30227</v>
+      </c>
+      <c r="B795" s="2" t="n">
+        <v>29.03</v>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" t="n">
+        <v>30228</v>
+      </c>
+      <c r="B796" s="5" t="n">
+        <v>3.02</v>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" t="n">
+        <v>30229</v>
+      </c>
+      <c r="B797" s="3" t="n">
+        <v>0.27</v>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" t="n">
+        <v>30230</v>
+      </c>
+      <c r="B798" s="5" t="n">
+        <v>3.27</v>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" t="n">
+        <v>30231</v>
+      </c>
+      <c r="B799" s="3" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" t="n">
+        <v>30232</v>
+      </c>
+      <c r="B800" s="4" t="n">
+        <v>5.48</v>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" t="n">
+        <v>30233</v>
+      </c>
+      <c r="B801" s="4" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" t="n">
+        <v>30234</v>
+      </c>
+      <c r="B802" s="3" t="n">
+        <v>2.72</v>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" t="n">
+        <v>30235</v>
+      </c>
+      <c r="B803" s="3" t="n">
+        <v>1.92</v>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" t="n">
+        <v>30236</v>
+      </c>
+      <c r="B804" s="3" t="n">
+        <v>2.41</v>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" t="n">
+        <v>30237</v>
+      </c>
+      <c r="B805" s="5" t="n">
+        <v>4.3</v>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" t="n">
+        <v>30238</v>
+      </c>
+      <c r="B806" s="3" t="n">
+        <v>2.96</v>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" t="n">
+        <v>30239</v>
+      </c>
+      <c r="B807" s="3" t="n">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" t="n">
+        <v>30240</v>
+      </c>
+      <c r="B808" s="3" t="n">
+        <v>1.57</v>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" t="n">
+        <v>30241</v>
+      </c>
+      <c r="B809" s="4" t="n">
+        <v>5.41</v>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" t="n">
+        <v>30242</v>
+      </c>
+      <c r="B810" s="5" t="n">
+        <v>3.27</v>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" t="n">
+        <v>30243</v>
+      </c>
+      <c r="B811" s="5" t="n">
+        <v>4.73</v>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" t="n">
+        <v>30244</v>
+      </c>
+      <c r="B812" s="2" t="n">
+        <v>9.1</v>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" t="n">
+        <v>30245</v>
+      </c>
+      <c r="B813" s="3" t="n">
+        <v>1.97</v>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" t="n">
+        <v>30246</v>
+      </c>
+      <c r="B814" s="3" t="n">
+        <v>1.03</v>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" t="n">
+        <v>30247</v>
+      </c>
+      <c r="B815" s="2" t="n">
+        <v>7.41</v>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" t="n">
+        <v>30248</v>
+      </c>
+      <c r="B816" s="3" t="n">
+        <v>1.62</v>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" t="n">
+        <v>30249</v>
+      </c>
+      <c r="B817" s="3" t="n">
+        <v>1.76</v>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" t="n">
+        <v>30250</v>
+      </c>
+      <c r="B818" s="4" t="n">
+        <v>6.42</v>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" t="n">
+        <v>30251</v>
+      </c>
+      <c r="B819" s="3" t="n">
+        <v>2.84</v>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" t="n">
+        <v>30252</v>
+      </c>
+      <c r="B820" s="3" t="n">
+        <v>2.53</v>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" t="n">
+        <v>30253</v>
+      </c>
+      <c r="B821" s="5" t="n">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" t="n">
+        <v>30254</v>
+      </c>
+      <c r="B822" s="5" t="n">
+        <v>4.66</v>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" t="n">
+        <v>30255</v>
+      </c>
+      <c r="B823" s="2" t="n">
+        <v>7.86</v>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" t="n">
+        <v>30256</v>
+      </c>
+      <c r="B824" s="5" t="n">
+        <v>4.46</v>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" t="n">
+        <v>30257</v>
+      </c>
+      <c r="B825" s="3" t="n">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" t="n">
+        <v>30258</v>
+      </c>
+      <c r="B826" s="3" t="n">
+        <v>0.99</v>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" t="n">
+        <v>30259</v>
+      </c>
+      <c r="B827" s="2" t="n">
+        <v>24.58</v>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" t="n">
+        <v>30260</v>
+      </c>
+      <c r="B828" s="2" t="n">
+        <v>8.32</v>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" t="n">
+        <v>30261</v>
+      </c>
+      <c r="B829" s="5" t="n">
+        <v>3.23</v>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" t="n">
+        <v>30262</v>
+      </c>
+      <c r="B830" s="5" t="n">
+        <v>4.67</v>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" t="n">
+        <v>30263</v>
+      </c>
+      <c r="B831" s="4" t="n">
+        <v>6.59</v>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" t="n">
+        <v>30264</v>
+      </c>
+      <c r="B832" s="2" t="n">
+        <v>11.46</v>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" t="n">
+        <v>30265</v>
+      </c>
+      <c r="B833" s="5" t="n">
+        <v>4.85</v>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" t="n">
+        <v>30266</v>
+      </c>
+      <c r="B834" s="2" t="n">
+        <v>9.09</v>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" t="n">
+        <v>30267</v>
+      </c>
+      <c r="B835" s="5" t="n">
+        <v>3.82</v>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" t="n">
+        <v>30268</v>
+      </c>
+      <c r="B836" s="2" t="n">
+        <v>7.51</v>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" t="n">
+        <v>30269</v>
+      </c>
+      <c r="B837" s="5" t="n">
+        <v>3.85</v>
+      </c>
+    </row>
+    <row r="838">
+      <c r="A838" t="n">
+        <v>30270</v>
+      </c>
+      <c r="B838" s="5" t="n">
+        <v>4.26</v>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" t="n">
+        <v>30271</v>
+      </c>
+      <c r="B839" s="5" t="n">
+        <v>4.16</v>
+      </c>
+    </row>
+    <row r="840">
+      <c r="A840" t="n">
+        <v>30272</v>
+      </c>
+      <c r="B840" s="3" t="n">
+        <v>1.99</v>
+      </c>
+    </row>
+    <row r="841">
+      <c r="A841" t="n">
+        <v>30273</v>
+      </c>
+      <c r="B841" s="3" t="n">
+        <v>2.49</v>
+      </c>
+    </row>
+    <row r="842">
+      <c r="A842" t="n">
+        <v>30274</v>
+      </c>
+      <c r="B842" s="5" t="n">
+        <v>3.73</v>
+      </c>
+    </row>
+    <row r="843">
+      <c r="A843" t="n">
+        <v>30275</v>
+      </c>
+      <c r="B843" s="3" t="n">
+        <v>2.3</v>
+      </c>
+    </row>
+    <row r="844">
+      <c r="A844" t="n">
+        <v>30276</v>
+      </c>
+      <c r="B844" s="5" t="n">
+        <v>4.44</v>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" t="n">
+        <v>30277</v>
+      </c>
+      <c r="B845" s="3" t="n">
+        <v>2.22</v>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" t="n">
+        <v>30278</v>
+      </c>
+      <c r="B846" s="3" t="n">
+        <v>2.58</v>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" t="n">
+        <v>30279</v>
+      </c>
+      <c r="B847" s="5" t="n">
+        <v>4.96</v>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" t="n">
+        <v>30280</v>
+      </c>
+      <c r="B848" s="5" t="n">
+        <v>3.95</v>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" t="n">
+        <v>30281</v>
+      </c>
+      <c r="B849" s="3" t="n">
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" t="n">
+        <v>30282</v>
+      </c>
+      <c r="B850" s="5" t="n">
+        <v>3.32</v>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" t="n">
+        <v>30283</v>
+      </c>
+      <c r="B851" s="2" t="n">
+        <v>8.74</v>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" t="n">
+        <v>30284</v>
+      </c>
+      <c r="B852" s="2" t="n">
+        <v>34.9</v>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" t="n">
+        <v>30285</v>
+      </c>
+      <c r="B853" s="3" t="n">
+        <v>2.38</v>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" t="n">
+        <v>30286</v>
+      </c>
+      <c r="B854" s="4" t="n">
+        <v>5.49</v>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" t="n">
+        <v>30287</v>
+      </c>
+      <c r="B855" s="5" t="n">
+        <v>3.36</v>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" t="n">
+        <v>30288</v>
+      </c>
+      <c r="B856" s="3" t="n">
+        <v>2.95</v>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" t="n">
+        <v>30289</v>
+      </c>
+      <c r="B857" s="4" t="n">
+        <v>5.12</v>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" t="n">
+        <v>30290</v>
+      </c>
+      <c r="B858" s="4" t="n">
+        <v>5.97</v>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" t="n">
+        <v>30291</v>
+      </c>
+      <c r="B859" s="2" t="n">
+        <v>8.77</v>
+      </c>
+    </row>
+    <row r="860">
+      <c r="A860" t="n">
+        <v>30292</v>
+      </c>
+      <c r="B860" s="2" t="n">
+        <v>11.36</v>
+      </c>
+    </row>
+    <row r="861">
+      <c r="A861" t="n">
+        <v>30293</v>
+      </c>
+      <c r="B861" s="4" t="n">
+        <v>6.6</v>
+      </c>
+    </row>
+    <row r="862">
+      <c r="A862" t="n">
+        <v>30294</v>
+      </c>
+      <c r="B862" s="5" t="n">
+        <v>4.9</v>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" t="n">
+        <v>30295</v>
+      </c>
+      <c r="B863" s="3" t="n">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" t="n">
+        <v>30296</v>
+      </c>
+      <c r="B864" s="3" t="n">
+        <v>1.26</v>
+      </c>
+    </row>
+    <row r="865">
+      <c r="A865" t="n">
+        <v>30297</v>
+      </c>
+      <c r="B865" s="3" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="866">
+      <c r="A866" t="n">
+        <v>30298</v>
+      </c>
+      <c r="B866" s="3" t="n">
+        <v>0.76</v>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" t="n">
+        <v>30299</v>
+      </c>
+      <c r="B867" s="3" t="n">
+        <v>0.91</v>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" t="n">
+        <v>30300</v>
+      </c>
+      <c r="B868" s="2" t="n">
+        <v>12.81</v>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" t="n">
+        <v>30301</v>
+      </c>
+      <c r="B869" s="3" t="n">
+        <v>1.87</v>
+      </c>
+    </row>
+    <row r="870">
+      <c r="A870" t="n">
+        <v>30302</v>
+      </c>
+      <c r="B870" s="4" t="n">
+        <v>5.31</v>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" t="n">
+        <v>30303</v>
+      </c>
+      <c r="B871" s="4" t="n">
+        <v>5.89</v>
+      </c>
+    </row>
+    <row r="872">
+      <c r="A872" t="n">
+        <v>30304</v>
+      </c>
+      <c r="B872" s="3" t="n">
+        <v>2.76</v>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" t="n">
+        <v>30305</v>
+      </c>
+      <c r="B873" s="3" t="n">
+        <v>1.44</v>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" t="n">
+        <v>30306</v>
+      </c>
+      <c r="B874" s="4" t="n">
+        <v>5.1</v>
+      </c>
+    </row>
+    <row r="875">
+      <c r="A875" t="n">
+        <v>30307</v>
+      </c>
+      <c r="B875" s="5" t="n">
+        <v>4.43</v>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" t="n">
+        <v>30308</v>
+      </c>
+      <c r="B876" s="3" t="n">
+        <v>2.84</v>
+      </c>
+    </row>
+    <row r="877">
+      <c r="A877" t="n">
+        <v>30309</v>
+      </c>
+      <c r="B877" s="4" t="n">
+        <v>5.44</v>
+      </c>
+    </row>
+    <row r="878">
+      <c r="A878" t="n">
+        <v>30310</v>
+      </c>
+      <c r="B878" s="3" t="n">
+        <v>2.18</v>
+      </c>
+    </row>
+    <row r="879">
+      <c r="A879" t="n">
+        <v>30311</v>
+      </c>
+      <c r="B879" s="3" t="n">
+        <v>1.14</v>
+      </c>
+    </row>
+    <row r="880">
+      <c r="A880" t="n">
+        <v>30312</v>
+      </c>
+      <c r="B880" s="3" t="n">
+        <v>1.95</v>
+      </c>
+    </row>
+    <row r="881">
+      <c r="A881" t="n">
+        <v>30313</v>
+      </c>
+      <c r="B881" s="5" t="n">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="882">
+      <c r="A882" t="n">
+        <v>30314</v>
+      </c>
+      <c r="B882" s="5" t="n">
+        <v>3.19</v>
+      </c>
+    </row>
+    <row r="883">
+      <c r="A883" t="n">
+        <v>30315</v>
+      </c>
+      <c r="B883" s="3" t="n">
+        <v>1.89</v>
+      </c>
+    </row>
+    <row r="884">
+      <c r="A884" t="n">
+        <v>30316</v>
+      </c>
+      <c r="B884" s="3" t="n">
+        <v>0.84</v>
+      </c>
+    </row>
+    <row r="885">
+      <c r="A885" t="n">
+        <v>30317</v>
+      </c>
+      <c r="B885" s="5" t="n">
+        <v>3.76</v>
+      </c>
+    </row>
+    <row r="886">
+      <c r="A886" t="n">
+        <v>30318</v>
+      </c>
+      <c r="B886" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="887">
+      <c r="A887" t="n">
+        <v>30319</v>
+      </c>
+      <c r="B887" s="3" t="n">
+        <v>2.17</v>
+      </c>
+    </row>
+    <row r="888">
+      <c r="A888" t="n">
+        <v>30320</v>
+      </c>
+      <c r="B888" s="3" t="n">
+        <v>2.3</v>
+      </c>
+    </row>
+    <row r="889">
+      <c r="A889" t="n">
+        <v>30321</v>
+      </c>
+      <c r="B889" s="3" t="n">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="890">
+      <c r="A890" t="n">
+        <v>30322</v>
+      </c>
+      <c r="B890" s="3" t="n">
+        <v>1.71</v>
+      </c>
+    </row>
+    <row r="891">
+      <c r="A891" t="n">
+        <v>30323</v>
+      </c>
+      <c r="B891" s="5" t="n">
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="892">
+      <c r="A892" t="n">
+        <v>30324</v>
+      </c>
+      <c r="B892" s="5" t="n">
+        <v>4.61</v>
+      </c>
+    </row>
+    <row r="893">
+      <c r="A893" t="n">
+        <v>30325</v>
+      </c>
+      <c r="B893" s="3" t="n">
+        <v>0.47</v>
+      </c>
+    </row>
+    <row r="894">
+      <c r="A894" t="n">
+        <v>30326</v>
+      </c>
+      <c r="B894" s="5" t="n">
+        <v>3.17</v>
+      </c>
+    </row>
+    <row r="895">
+      <c r="A895" t="n">
+        <v>30327</v>
+      </c>
+      <c r="B895" s="3" t="n">
+        <v>2.61</v>
+      </c>
+    </row>
+    <row r="896">
+      <c r="A896" t="n">
+        <v>30328</v>
+      </c>
+      <c r="B896" s="3" t="n">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="897">
+      <c r="A897" t="n">
+        <v>30329</v>
+      </c>
+      <c r="B897" s="4" t="n">
+        <v>5.25</v>
+      </c>
+    </row>
+    <row r="898">
+      <c r="A898" t="n">
+        <v>30330</v>
+      </c>
+      <c r="B898" s="3" t="n">
+        <v>2.06</v>
+      </c>
+    </row>
+    <row r="899">
+      <c r="A899" t="n">
+        <v>30331</v>
+      </c>
+      <c r="B899" s="5" t="n">
+        <v>3.16</v>
+      </c>
+    </row>
+    <row r="900">
+      <c r="A900" t="n">
+        <v>30332</v>
+      </c>
+      <c r="B900" s="2" t="n">
+        <v>8.59</v>
+      </c>
+    </row>
+    <row r="901">
+      <c r="A901" t="n">
+        <v>30333</v>
+      </c>
+      <c r="B901" s="3" t="n">
+        <v>2.57</v>
+      </c>
+    </row>
+    <row r="902">
+      <c r="A902" t="n">
+        <v>30334</v>
+      </c>
+      <c r="B902" s="2" t="n">
+        <v>101.59</v>
+      </c>
+    </row>
+    <row r="903">
+      <c r="A903" t="n">
+        <v>30335</v>
+      </c>
+      <c r="B903" s="3" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="904">
+      <c r="A904" t="n">
+        <v>30336</v>
+      </c>
+      <c r="B904" s="3" t="n">
+        <v>2.54</v>
+      </c>
+    </row>
+    <row r="905">
+      <c r="A905" t="n">
+        <v>30337</v>
+      </c>
+      <c r="B905" s="5" t="n">
+        <v>3.03</v>
+      </c>
+    </row>
+    <row r="906">
+      <c r="A906" t="n">
+        <v>30338</v>
+      </c>
+      <c r="B906" s="3" t="n">
+        <v>2.94</v>
+      </c>
+    </row>
+    <row r="907">
+      <c r="A907" t="n">
+        <v>30339</v>
+      </c>
+      <c r="B907" s="3" t="n">
+        <v>2.72</v>
+      </c>
+    </row>
+    <row r="908">
+      <c r="A908" t="n">
+        <v>30340</v>
+      </c>
+      <c r="B908" s="5" t="n">
+        <v>3.26</v>
+      </c>
+    </row>
+    <row r="909">
+      <c r="A909" t="n">
+        <v>30341</v>
+      </c>
+      <c r="B909" s="3" t="n">
+        <v>2.84</v>
+      </c>
+    </row>
+    <row r="910">
+      <c r="A910" t="n">
+        <v>30342</v>
+      </c>
+      <c r="B910" s="3" t="n">
+        <v>1.76</v>
+      </c>
+    </row>
+    <row r="911">
+      <c r="A911" t="n">
+        <v>30343</v>
+      </c>
+      <c r="B911" s="5" t="n">
+        <v>3.42</v>
+      </c>
+    </row>
+    <row r="912">
+      <c r="A912" t="n">
+        <v>30344</v>
+      </c>
+      <c r="B912" s="3" t="n">
+        <v>2.84</v>
+      </c>
+    </row>
+    <row r="913">
+      <c r="A913" t="n">
+        <v>30345</v>
+      </c>
+      <c r="B913" s="5" t="n">
+        <v>3.93</v>
+      </c>
+    </row>
+    <row r="914">
+      <c r="A914" t="n">
+        <v>30346</v>
+      </c>
+      <c r="B914" s="4" t="n">
+        <v>6.39</v>
+      </c>
+    </row>
+    <row r="915">
+      <c r="A915" t="n">
+        <v>30347</v>
+      </c>
+      <c r="B915" s="4" t="n">
+        <v>5.18</v>
+      </c>
+    </row>
+    <row r="916">
+      <c r="A916" t="n">
+        <v>30348</v>
+      </c>
+      <c r="B916" s="5" t="n">
+        <v>4.69</v>
+      </c>
+    </row>
+    <row r="917">
+      <c r="A917" t="n">
+        <v>30349</v>
+      </c>
+      <c r="B917" s="3" t="n">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="918">
+      <c r="A918" t="n">
+        <v>30350</v>
+      </c>
+      <c r="B918" s="3" t="n">
+        <v>2.05</v>
+      </c>
+    </row>
+    <row r="919">
+      <c r="A919" t="n">
+        <v>30351</v>
+      </c>
+      <c r="B919" s="2" t="n">
+        <v>21.66</v>
+      </c>
+    </row>
+    <row r="920">
+      <c r="A920" t="n">
+        <v>30352</v>
+      </c>
+      <c r="B920" s="3" t="n">
+        <v>2.69</v>
+      </c>
+    </row>
+    <row r="921">
+      <c r="A921" t="n">
+        <v>30353</v>
+      </c>
+      <c r="B921" s="2" t="n">
+        <v>9.35</v>
+      </c>
+    </row>
+    <row r="922">
+      <c r="A922" t="n">
+        <v>30354</v>
+      </c>
+      <c r="B922" s="5" t="n">
+        <v>3.32</v>
+      </c>
+    </row>
+    <row r="923">
+      <c r="A923" t="n">
+        <v>30355</v>
+      </c>
+      <c r="B923" s="3" t="n">
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="924">
+      <c r="A924" t="n">
+        <v>30356</v>
+      </c>
+      <c r="B924" s="3" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+    </row>
+    <row r="925">
+      <c r="A925" t="n">
+        <v>30357</v>
+      </c>
+      <c r="B925" s="3" t="n">
+        <v>0.97</v>
+      </c>
+    </row>
+    <row r="926">
+      <c r="A926" t="n">
+        <v>30358</v>
+      </c>
+      <c r="B926" s="3" t="n">
+        <v>1.88</v>
+      </c>
+    </row>
+    <row r="927">
+      <c r="A927" t="n">
+        <v>30359</v>
+      </c>
+      <c r="B927" s="3" t="n">
+        <v>2.64</v>
+      </c>
+    </row>
+    <row r="928">
+      <c r="A928" t="n">
+        <v>30360</v>
+      </c>
+      <c r="B928" s="5" t="n">
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="929">
+      <c r="A929" t="n">
+        <v>30361</v>
+      </c>
+      <c r="B929" s="3" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="930">
+      <c r="A930" t="n">
+        <v>30362</v>
+      </c>
+      <c r="B930" s="3" t="n">
+        <v>2.3</v>
+      </c>
+    </row>
+    <row r="931">
+      <c r="A931" t="n">
+        <v>30363</v>
+      </c>
+      <c r="B931" s="2" t="n">
+        <v>7.42</v>
+      </c>
+    </row>
+    <row r="932">
+      <c r="A932" t="n">
+        <v>30364</v>
+      </c>
+      <c r="B932" s="5" t="n">
+        <v>4.86</v>
+      </c>
+    </row>
+    <row r="933">
+      <c r="A933" t="n">
+        <v>30365</v>
+      </c>
+      <c r="B933" s="2" t="n">
+        <v>7.27</v>
+      </c>
+    </row>
+    <row r="934">
+      <c r="A934" t="n">
+        <v>30366</v>
+      </c>
+      <c r="B934" s="2" t="n">
+        <v>8.44</v>
+      </c>
+    </row>
+    <row r="935">
+      <c r="A935" t="n">
+        <v>30367</v>
+      </c>
+      <c r="B935" s="4" t="n">
+        <v>6.54</v>
+      </c>
+    </row>
+    <row r="936">
+      <c r="A936" t="n">
+        <v>30368</v>
+      </c>
+      <c r="B936" s="5" t="n">
+        <v>4.19</v>
+      </c>
+    </row>
+    <row r="937">
+      <c r="A937" t="n">
+        <v>30369</v>
+      </c>
+      <c r="B937" s="5" t="n">
+        <v>4.29</v>
+      </c>
+    </row>
+    <row r="938">
+      <c r="A938" t="n">
+        <v>30370</v>
+      </c>
+      <c r="B938" s="2" t="n">
+        <v>7.28</v>
+      </c>
+    </row>
+    <row r="939">
+      <c r="A939" t="n">
+        <v>30371</v>
+      </c>
+      <c r="B939" s="2" t="n">
+        <v>11.25</v>
+      </c>
+    </row>
+    <row r="940">
+      <c r="A940" t="n">
+        <v>30372</v>
+      </c>
+      <c r="B940" s="5" t="n">
+        <v>4.56</v>
+      </c>
+    </row>
+    <row r="941">
+      <c r="A941" t="n">
+        <v>30373</v>
+      </c>
+      <c r="B941" s="5" t="n">
+        <v>3.41</v>
+      </c>
+    </row>
+    <row r="942">
+      <c r="A942" t="n">
+        <v>30374</v>
+      </c>
+      <c r="B942" s="2" t="n">
+        <v>7.26</v>
+      </c>
+    </row>
+    <row r="943">
+      <c r="A943" t="n">
+        <v>30375</v>
+      </c>
+      <c r="B943" s="4" t="n">
+        <v>5.38</v>
+      </c>
+    </row>
+    <row r="944">
+      <c r="A944" t="n">
+        <v>30376</v>
+      </c>
+      <c r="B944" s="3" t="n">
+        <v>1.84</v>
+      </c>
+    </row>
+    <row r="945">
+      <c r="A945" t="n">
+        <v>30377</v>
+      </c>
+      <c r="B945" s="5" t="n">
+        <v>4.92</v>
+      </c>
+    </row>
+    <row r="946">
+      <c r="A946" t="n">
+        <v>30378</v>
+      </c>
+      <c r="B946" s="5" t="n">
+        <v>4.91</v>
+      </c>
+    </row>
+    <row r="947">
+      <c r="A947" t="n">
+        <v>30379</v>
+      </c>
+      <c r="B947" s="3" t="n">
+        <v>1.78</v>
+      </c>
+    </row>
+    <row r="948">
+      <c r="A948" t="n">
+        <v>30380</v>
+      </c>
+      <c r="B948" s="2" t="n">
+        <v>9.23</v>
+      </c>
+    </row>
+    <row r="949">
+      <c r="A949" t="n">
+        <v>30381</v>
+      </c>
+      <c r="B949" s="2" t="n">
+        <v>16.75</v>
+      </c>
+    </row>
+    <row r="950">
+      <c r="A950" t="n">
+        <v>30382</v>
+      </c>
+      <c r="B950" s="3" t="n">
+        <v>1.39</v>
+      </c>
+    </row>
+    <row r="951">
+      <c r="A951" t="n">
+        <v>30383</v>
+      </c>
+      <c r="B951" s="3" t="n">
+        <v>2.32</v>
+      </c>
+    </row>
+    <row r="952">
+      <c r="A952" t="n">
+        <v>30384</v>
+      </c>
+      <c r="B952" s="3" t="n">
+        <v>2.75</v>
+      </c>
+    </row>
+    <row r="953">
+      <c r="A953" t="n">
+        <v>30385</v>
+      </c>
+      <c r="B953" s="3" t="n">
+        <v>2.85</v>
+      </c>
+    </row>
+    <row r="954">
+      <c r="A954" t="n">
+        <v>30386</v>
+      </c>
+      <c r="B954" s="3" t="n">
+        <v>2.95</v>
+      </c>
+    </row>
+    <row r="955">
+      <c r="A955" t="n">
+        <v>30387</v>
+      </c>
+      <c r="B955" s="3" t="n">
+        <v>2.26</v>
+      </c>
+    </row>
+    <row r="956">
+      <c r="A956" t="n">
+        <v>30388</v>
+      </c>
+      <c r="B956" s="5" t="n">
+        <v>4.44</v>
+      </c>
+    </row>
+    <row r="957">
+      <c r="A957" t="n">
+        <v>30389</v>
+      </c>
+      <c r="B957" s="4" t="n">
+        <v>6.01</v>
+      </c>
+    </row>
+    <row r="958">
+      <c r="A958" t="n">
+        <v>30390</v>
+      </c>
+      <c r="B958" s="5" t="n">
+        <v>3.52</v>
+      </c>
+    </row>
+    <row r="959">
+      <c r="A959" t="n">
+        <v>30391</v>
+      </c>
+      <c r="B959" s="2" t="n">
+        <v>7.11</v>
+      </c>
+    </row>
+    <row r="960">
+      <c r="A960" t="n">
+        <v>30392</v>
+      </c>
+      <c r="B960" s="4" t="n">
+        <v>6.4</v>
+      </c>
+    </row>
+    <row r="961">
+      <c r="A961" t="n">
+        <v>30393</v>
+      </c>
+      <c r="B961" s="5" t="n">
+        <v>3.99</v>
+      </c>
+    </row>
+    <row r="962">
+      <c r="A962" t="n">
+        <v>30394</v>
+      </c>
+      <c r="B962" s="2" t="n">
+        <v>23.65</v>
+      </c>
+    </row>
+    <row r="963">
+      <c r="A963" t="n">
+        <v>30395</v>
+      </c>
+      <c r="B963" s="5" t="n">
+        <v>4.05</v>
+      </c>
+    </row>
+    <row r="964">
+      <c r="A964" t="n">
+        <v>30396</v>
+      </c>
+      <c r="B964" s="3" t="n">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="965">
+      <c r="A965" t="n">
+        <v>30397</v>
+      </c>
+      <c r="B965" s="5" t="n">
+        <v>3.13</v>
+      </c>
+    </row>
+    <row r="966">
+      <c r="A966" t="n">
+        <v>30398</v>
+      </c>
+      <c r="B966" s="2" t="n">
+        <v>14.59</v>
+      </c>
+    </row>
+    <row r="967">
+      <c r="A967" t="n">
+        <v>30399</v>
+      </c>
+      <c r="B967" s="3" t="n">
+        <v>1.16</v>
+      </c>
+    </row>
+    <row r="968">
+      <c r="A968" t="n">
+        <v>30400</v>
+      </c>
+      <c r="B968" s="3" t="n">
+        <v>2.96</v>
+      </c>
+    </row>
+    <row r="969">
+      <c r="A969" t="n">
+        <v>30401</v>
+      </c>
+      <c r="B969" s="3" t="n">
+        <v>1.19</v>
+      </c>
+    </row>
+    <row r="970">
+      <c r="A970" t="n">
+        <v>30402</v>
+      </c>
+      <c r="B970" s="2" t="n">
+        <v>9.220000000000001</v>
+      </c>
+    </row>
+    <row r="971">
+      <c r="A971" t="n">
+        <v>30403</v>
+      </c>
+      <c r="B971" s="5" t="n">
+        <v>3.19</v>
+      </c>
+    </row>
+    <row r="972">
+      <c r="A972" t="n">
+        <v>30404</v>
+      </c>
+      <c r="B972" s="3" t="n">
+        <v>1.53</v>
+      </c>
+    </row>
+    <row r="973">
+      <c r="A973" t="n">
+        <v>30405</v>
+      </c>
+      <c r="B973" s="2" t="n">
+        <v>9.130000000000001</v>
+      </c>
+    </row>
+    <row r="974">
+      <c r="A974" t="n">
+        <v>30406</v>
+      </c>
+      <c r="B974" s="2" t="n">
+        <v>7.45</v>
+      </c>
+    </row>
+    <row r="975">
+      <c r="A975" t="n">
+        <v>30407</v>
+      </c>
+      <c r="B975" s="3" t="n">
+        <v>1.38</v>
+      </c>
+    </row>
+    <row r="976">
+      <c r="A976" t="n">
+        <v>30408</v>
+      </c>
+      <c r="B976" s="4" t="n">
+        <v>5.57</v>
+      </c>
+    </row>
+    <row r="977">
+      <c r="A977" t="n">
+        <v>30409</v>
+      </c>
+      <c r="B977" s="3" t="n">
+        <v>1.52</v>
+      </c>
+    </row>
+    <row r="978">
+      <c r="A978" t="n">
+        <v>30410</v>
+      </c>
+      <c r="B978" s="3" t="n">
+        <v>2.3</v>
+      </c>
+    </row>
+    <row r="979">
+      <c r="A979" t="n">
+        <v>30411</v>
+      </c>
+      <c r="B979" s="2" t="n">
+        <v>7.37</v>
+      </c>
+    </row>
+    <row r="980">
+      <c r="A980" t="n">
+        <v>30412</v>
+      </c>
+      <c r="B980" s="3" t="n">
+        <v>1.91</v>
+      </c>
+    </row>
+    <row r="981">
+      <c r="A981" t="n">
+        <v>30413</v>
+      </c>
+      <c r="B981" s="4" t="n">
+        <v>6.21</v>
+      </c>
+    </row>
+    <row r="982">
+      <c r="A982" t="n">
+        <v>30414</v>
+      </c>
+      <c r="B982" s="5" t="n">
+        <v>3.95</v>
+      </c>
+    </row>
+    <row r="983">
+      <c r="A983" t="n">
+        <v>30415</v>
+      </c>
+      <c r="B983" s="3" t="n">
+        <v>2.81</v>
+      </c>
+    </row>
+    <row r="984">
+      <c r="A984" t="n">
+        <v>30416</v>
+      </c>
+      <c r="B984" s="2" t="n">
+        <v>12.28</v>
+      </c>
+    </row>
+    <row r="985">
+      <c r="A985" t="n">
+        <v>30417</v>
+      </c>
+      <c r="B985" s="3" t="n">
+        <v>0.76</v>
+      </c>
+    </row>
+    <row r="986">
+      <c r="A986" t="n">
+        <v>30418</v>
+      </c>
+      <c r="B986" s="5" t="n">
+        <v>3.27</v>
+      </c>
+    </row>
+    <row r="987">
+      <c r="A987" t="n">
+        <v>30419</v>
+      </c>
+      <c r="B987" s="3" t="n">
+        <v>2.26</v>
+      </c>
+    </row>
+    <row r="988">
+      <c r="A988" t="n">
+        <v>30420</v>
+      </c>
+      <c r="B988" s="3" t="n">
+        <v>2.08</v>
+      </c>
+    </row>
+    <row r="989">
+      <c r="A989" t="n">
+        <v>30421</v>
+      </c>
+      <c r="B989" s="3" t="n">
+        <v>0.91</v>
+      </c>
+    </row>
+    <row r="990">
+      <c r="A990" t="n">
+        <v>30422</v>
+      </c>
+      <c r="B990" s="5" t="n">
+        <v>3.06</v>
+      </c>
+    </row>
+    <row r="991">
+      <c r="A991" t="n">
+        <v>30423</v>
+      </c>
+      <c r="B991" s="3" t="n">
+        <v>1.58</v>
+      </c>
+    </row>
+    <row r="992">
+      <c r="A992" t="n">
+        <v>30424</v>
+      </c>
+      <c r="B992" s="4" t="n">
+        <v>6.29</v>
+      </c>
+    </row>
+    <row r="993">
+      <c r="A993" t="n">
+        <v>30425</v>
+      </c>
+      <c r="B993" s="5" t="n">
+        <v>3.45</v>
+      </c>
+    </row>
+    <row r="994">
+      <c r="A994" t="n">
+        <v>30426</v>
+      </c>
+      <c r="B994" s="3" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="995">
+      <c r="A995" t="n">
+        <v>30427</v>
+      </c>
+      <c r="B995" s="3" t="n">
+        <v>2.04</v>
+      </c>
+    </row>
+    <row r="996">
+      <c r="A996" t="n">
+        <v>30428</v>
+      </c>
+      <c r="B996" s="4" t="n">
+        <v>6.43</v>
+      </c>
+    </row>
+    <row r="997">
+      <c r="A997" t="n">
+        <v>30429</v>
+      </c>
+      <c r="B997" s="2" t="n">
+        <v>7.05</v>
+      </c>
+    </row>
+    <row r="998">
+      <c r="A998" t="n">
+        <v>30430</v>
+      </c>
+      <c r="B998" s="3" t="n">
+        <v>2.84</v>
+      </c>
+    </row>
+    <row r="999">
+      <c r="A999" t="n">
+        <v>30431</v>
+      </c>
+      <c r="B999" s="3" t="n">
+        <v>1.04</v>
+      </c>
+    </row>
+    <row r="1000">
+      <c r="A1000" t="n">
+        <v>30432</v>
+      </c>
+      <c r="B1000" s="3" t="n">
+        <v>1.53</v>
+      </c>
+    </row>
+    <row r="1001">
+      <c r="A1001" t="n">
+        <v>30433</v>
+      </c>
+      <c r="B1001" s="4" t="n">
+        <v>6.12</v>
+      </c>
+    </row>
+    <row r="1002">
+      <c r="A1002" t="n">
+        <v>30434</v>
+      </c>
+      <c r="B1002" s="2" t="n">
+        <v>10.49</v>
+      </c>
+    </row>
+    <row r="1003">
+      <c r="A1003" t="n">
+        <v>30435</v>
+      </c>
+      <c r="B1003" s="3" t="n">
+        <v>2.49</v>
+      </c>
+    </row>
+    <row r="1004">
+      <c r="A1004" t="n">
+        <v>30436</v>
+      </c>
+      <c r="B1004" s="3" t="n">
+        <v>1.92</v>
+      </c>
+    </row>
+    <row r="1005">
+      <c r="A1005" t="n">
+        <v>30437</v>
+      </c>
+      <c r="B1005" s="3" t="n">
+        <v>1.06</v>
+      </c>
+    </row>
+    <row r="1006">
+      <c r="A1006" t="n">
+        <v>30438</v>
+      </c>
+      <c r="B1006" s="5" t="n">
+        <v>4.83</v>
+      </c>
+    </row>
+    <row r="1007">
+      <c r="A1007" t="n">
+        <v>30439</v>
+      </c>
+      <c r="B1007" s="3" t="n">
+        <v>1.95</v>
+      </c>
+    </row>
+    <row r="1008">
+      <c r="A1008" t="n">
+        <v>30440</v>
+      </c>
+      <c r="B1008" s="3" t="n">
+        <v>1.27</v>
+      </c>
+    </row>
+    <row r="1009">
+      <c r="A1009" t="n">
+        <v>30441</v>
+      </c>
+      <c r="B1009" s="3" t="n">
+        <v>0.93</v>
+      </c>
+    </row>
+    <row r="1010">
+      <c r="A1010" t="n">
+        <v>30442</v>
+      </c>
+      <c r="B1010" s="3" t="n">
+        <v>1.24</v>
+      </c>
+    </row>
+    <row r="1011">
+      <c r="A1011" t="n">
+        <v>30443</v>
+      </c>
+      <c r="B1011" s="5" t="n">
+        <v>3.37</v>
+      </c>
+    </row>
+    <row r="1012">
+      <c r="A1012" t="n">
+        <v>30444</v>
+      </c>
+      <c r="B1012" s="2" t="n">
+        <v>7.83</v>
+      </c>
+    </row>
+    <row r="1013">
+      <c r="A1013" t="n">
+        <v>30445</v>
+      </c>
+      <c r="B1013" s="3" t="n">
+        <v>1.97</v>
+      </c>
+    </row>
+    <row r="1014">
+      <c r="A1014" t="n">
+        <v>30446</v>
+      </c>
+      <c r="B1014" s="3" t="n">
+        <v>2.07</v>
+      </c>
+    </row>
+    <row r="1015">
+      <c r="A1015" t="n">
+        <v>30447</v>
+      </c>
+      <c r="B1015" s="5" t="n">
+        <v>3.53</v>
+      </c>
+    </row>
+    <row r="1016">
+      <c r="A1016" t="n">
+        <v>30448</v>
+      </c>
+      <c r="B1016" s="5" t="n">
+        <v>3.59</v>
+      </c>
+    </row>
+    <row r="1017">
+      <c r="A1017" t="n">
+        <v>30449</v>
+      </c>
+      <c r="B1017" s="3" t="n">
+        <v>2.04</v>
+      </c>
+    </row>
+    <row r="1018">
+      <c r="A1018" t="n">
+        <v>30450</v>
+      </c>
+      <c r="B1018" s="3" t="n">
+        <v>1.35</v>
+      </c>
+    </row>
+    <row r="1019">
+      <c r="A1019" t="n">
+        <v>30451</v>
+      </c>
+      <c r="B1019" s="5" t="n">
+        <v>3.66</v>
+      </c>
+    </row>
+    <row r="1020">
+      <c r="A1020" t="n">
+        <v>30452</v>
+      </c>
+      <c r="B1020" s="3" t="n">
+        <v>2.54</v>
+      </c>
+    </row>
+    <row r="1021">
+      <c r="A1021" t="n">
+        <v>30453</v>
+      </c>
+      <c r="B1021" s="3" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="1022">
+      <c r="A1022" t="n">
+        <v>30454</v>
+      </c>
+      <c r="B1022" s="3" t="n">
+        <v>2.95</v>
+      </c>
+    </row>
+    <row r="1023">
+      <c r="A1023" t="n">
+        <v>30455</v>
+      </c>
+      <c r="B1023" s="3" t="n">
+        <v>1.47</v>
+      </c>
+    </row>
+    <row r="1024">
+      <c r="A1024" t="n">
+        <v>30456</v>
+      </c>
+      <c r="B1024" s="3" t="n">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="1025">
+      <c r="A1025" t="n">
+        <v>30458</v>
+      </c>
+      <c r="B1025" s="2" t="n">
+        <v>7.5</v>
+      </c>
+    </row>
+    <row r="1026">
+      <c r="A1026" t="n">
+        <v>30459</v>
+      </c>
+      <c r="B1026" s="4" t="n">
+        <v>5.53</v>
+      </c>
+    </row>
+    <row r="1027">
+      <c r="A1027" t="n">
+        <v>30460</v>
+      </c>
+      <c r="B1027" s="5" t="n">
+        <v>3.47</v>
+      </c>
+    </row>
+    <row r="1028">
+      <c r="A1028" t="n">
+        <v>30461</v>
+      </c>
+      <c r="B1028" s="3" t="n">
+        <v>1.41</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>